<commit_message>
feat: generate catalogs (carvings, graphics) and add JSON/images
</commit_message>
<xml_diff>
--- a/apps/bot/catalog.xlsx
+++ b/apps/bot/catalog.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB835AB-6003-47E5-96EB-87403328E789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE5BC3B-B546-42DF-B276-43A118E6C25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -421,12 +421,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -441,9 +447,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -815,182 +823,182 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="2">
         <v>10600</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="E2" s="2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>29200</v>
       </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="E7" s="2">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>39600</v>
       </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="E8" s="2">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1095,59 +1103,60 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="2">
         <v>13000</v>
       </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
+      <c r="E16" s="2">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="2">
         <v>13000</v>
       </c>
-      <c r="E17">
-        <v>1</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="E17" s="2">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="2">
         <v>15000</v>
       </c>
-      <c r="E18">
-        <v>1</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="E18" s="2">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1212,342 +1221,342 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
-        <v>1</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="D22" s="2">
+        <v>3600</v>
+      </c>
+      <c r="E22" s="2">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="A23" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23">
-        <v>1</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="D23" s="2">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="A24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D24">
-        <v>0</v>
-      </c>
-      <c r="E24">
-        <v>1</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="D24" s="2">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="A25" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25">
-        <v>1</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="D25" s="2">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="A26" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>1</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="D26" s="2">
+        <v>0</v>
+      </c>
+      <c r="E26" s="2">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="A27" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D27">
-        <v>0</v>
-      </c>
-      <c r="E27">
-        <v>1</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="D27" s="3">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3">
+        <v>1</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
+      <c r="A28" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-      <c r="E28">
-        <v>1</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="D28" s="3">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3">
+        <v>1</v>
+      </c>
+      <c r="F28" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="A29" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D29">
-        <v>0</v>
-      </c>
-      <c r="E29">
-        <v>1</v>
-      </c>
-      <c r="F29" t="s">
+      <c r="D29" s="3">
+        <v>0</v>
+      </c>
+      <c r="E29" s="3">
+        <v>1</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="A30" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D30">
-        <v>0</v>
-      </c>
-      <c r="E30">
-        <v>1</v>
-      </c>
-      <c r="F30" t="s">
+      <c r="D30" s="3">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="A31" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D31">
-        <v>0</v>
-      </c>
-      <c r="E31">
-        <v>1</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="D31" s="3">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3">
+        <v>1</v>
+      </c>
+      <c r="F31" s="3" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+      <c r="A32" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="2">
         <v>3500</v>
       </c>
-      <c r="E32">
-        <v>1</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="E32" s="2">
+        <v>1</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="A33" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="2">
         <v>1000</v>
       </c>
-      <c r="E33">
-        <v>1</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="E33" s="2">
+        <v>1</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
+      <c r="A34" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="3">
         <v>1000</v>
       </c>
-      <c r="E34">
-        <v>1</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="E34" s="3">
+        <v>1</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+      <c r="A35" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D35">
-        <v>0</v>
-      </c>
-      <c r="E35">
-        <v>1</v>
-      </c>
-      <c r="F35" t="s">
+      <c r="D35" s="3">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3">
+        <v>1</v>
+      </c>
+      <c r="F35" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
+      <c r="A36" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D36">
-        <v>0</v>
-      </c>
-      <c r="E36">
-        <v>1</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="D36" s="3">
+        <v>0</v>
+      </c>
+      <c r="E36" s="3">
+        <v>1</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+      <c r="A37" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D37">
-        <v>0</v>
-      </c>
-      <c r="E37">
-        <v>1</v>
-      </c>
-      <c r="F37" t="s">
+      <c r="D37" s="3">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3">
+        <v>1</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="A38" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="D38">
-        <v>0</v>
-      </c>
-      <c r="E38">
-        <v>1</v>
-      </c>
-      <c r="F38" t="s">
+      <c r="D38" s="3">
+        <v>0</v>
+      </c>
+      <c r="E38" s="3">
+        <v>1</v>
+      </c>
+      <c r="F38" s="3" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>